<commit_message>
feat: automação NFS-e SP com interface gráfica
</commit_message>
<xml_diff>
--- a/dados/sao_paulo/sao_paulo.xlsx
+++ b/dados/sao_paulo/sao_paulo.xlsx
@@ -8,27 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Contrato\Downloads\Data Dealer\automacao-nfs\dados\sao_paulo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA133B4-7A3E-4829-A2A2-17BB531DE0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C7D72D-33AB-460B-A5CB-C273DF58C1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1EA83C79-E727-4353-BA41-A0A665306418}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -37,9 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>https://nfe.prefeitura.sp.gov.br/login.aspx</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Data de Emissão</t>
+  </si>
+  <si>
+    <t>Valor</t>
   </si>
   <si>
     <t>Nome da Empresa</t>
@@ -51,31 +45,64 @@
     <t>Certificado Digital .PFX</t>
   </si>
   <si>
-    <t>Senha do Certificado</t>
-  </si>
-  <si>
-    <t>Tomador</t>
-  </si>
-  <si>
-    <t>CJPJ Tomador</t>
-  </si>
-  <si>
-    <t>Valor</t>
-  </si>
-  <si>
-    <t>Local da Prestação</t>
+    <t>Senha da Certidão</t>
+  </si>
+  <si>
+    <t>CNPJ Tomador</t>
+  </si>
+  <si>
+    <t>Observação</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>08/04/2026 17:15</t>
   </si>
   <si>
     <t>VALERIA MANEGEMENT</t>
   </si>
   <si>
-    <t>URL do Sistema</t>
+    <t>./dados/sao_paulo/certidoes/VALERIA CRISTINA DE PADUA.pfx</t>
+  </si>
+  <si>
+    <t>Valeria2026</t>
+  </si>
+  <si>
+    <t>33.512.889/0001-45</t>
+  </si>
+  <si>
+    <t>08/04/2026 17:00</t>
+  </si>
+  <si>
+    <t>CAROLINA</t>
+  </si>
+  <si>
+    <t>./dados/sao_paulo/certidoes/CAROLINA BARROS.pfx</t>
+  </si>
+  <si>
+    <t>Carolina2025</t>
+  </si>
+  <si>
+    <t>54.536.709/0001-35</t>
+  </si>
+  <si>
+    <t>MANA CONSULTORIA</t>
+  </si>
+  <si>
+    <t>./dados/sao_paulo/certidoes/PAULO HENRIQUE WODEWOTZKY LTDA_60720594000137.pfx</t>
+  </si>
+  <si>
+    <t>Paulo2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="00\.000\.000\/0000\-00"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -93,14 +120,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="7"/>
-      <color rgb="FF374151"/>
-      <name val="Courier New"/>
-      <family val="3"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <u/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -127,16 +155,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,17 +489,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A73E7066-E55D-4594-91F3-9F4B115F5217}">
-  <dimension ref="A1:J2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="9" width="20.109375" customWidth="1"/>
+    <col min="1" max="1" width="20.109375" customWidth="1"/>
+    <col min="2" max="3" width="18.109375" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="81.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="20.109375" customWidth="1"/>
+    <col min="9" max="9" width="23.5546875" customWidth="1"/>
+    <col min="10" max="10" width="27.88671875" customWidth="1"/>
+    <col min="11" max="11" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -471,7 +519,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -486,17 +534,140 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="6">
+        <v>53656846000140</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6">
+        <v>11735236000192</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="6">
+        <v>22121066000172</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="6">
+        <v>60720594000137</v>
+      </c>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="E5" s="6"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="E6" s="6"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E7" s="6"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E8" s="6"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E9" s="6"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E10" s="6"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E12" s="6"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E14" s="6"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E15" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>